<commit_message>
V-TOP Europe WPXA26B0912CZ320: use client's HS codes and Czech descriptions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pg2bih9dX5QihkKn7PSdjY
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
+++ b/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
@@ -102,6 +102,18 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -112,18 +124,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -521,25 +521,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="70" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,546 +631,614 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>HS kódy + popis</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Instrukce klienta – instrukce_18.9.2026.xlsx (zaslala Kateřina Buckingham)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Odesílatel</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>HS kód (TARIC)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Zdroj HS kódu</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Popis zboží (dle faktury – EN, CZ popis nedodán)</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Návrh CZ popisu (Claude – ke kontrole)</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Popis zboží (CZ – dle instrukce klienta)</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Položky (Ontime kód)</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Země původu</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Množství (ks)</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg) vč. palet</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Hodnota EUR (Total)</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>Clo třetí země</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>Melt &amp; pour</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t>Klasifikace – CCT/VPV KN tariff rule (CO / Z ČEHO / K ČEMU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ CCT/VPV KN tariff rule (odvozeno)</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>CLK872: CABLE LOCK-NEW-2A 58KHZ SUPER LOCK BLACK 175MM LENGTH 2 ALARAMS; HDL033-ST: BOTTLE TAG WITH METAL CABLE 160MM 58KHZ SUPER LOCK BLACK 160MM CABLE LENGTH WITH BLACK TUBE, WITH BLACK BALL; MINI PENCIL 50*14*20MM NORMAL LOCK 33MM FERRITE 58K GREY; HDP674-ST: PICCO 50 8.2MHZ SUPER LOCK WHITE 16MMS; HDL610: MICKEY PENCIL-B WITH LANYARD 8.2MHZ SUPER LOCK BLACK CABLE LENGTH 175MM 16MM GROOVED PIN; PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 2000PCS PER ROLL WITHOUT LOGO; PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 1000PCS PER ROLL WITHOUT LOGO; PL686: 3*3 ROLL LABEL 8.2MHZ WHITE DEACTIVABLE 1000PCS PER ROLL WITHOUT LOGO; ROUND RF LABEL 8.2MHZ WHITE DEACTIVABLE 1000PCS PER ROLL WITHOUT LOGO; PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 500PCS PER ROLL WITHOUT LOGO; SHELL TAG 58KHZ WHITE SL RED&amp;YELLOW INK(2 RED+1 YELLOW) 16MM SMOOTH PIN; AM LABEL 58KHZ BLACK DEACTIVATABLE</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Části elektrických signalizačních zařízení proti krádeži (EAS) – pevné ochranné štítky (AM 58 kHz / RF 8,2 MHz) a deaktivovatelné etikety</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>AS1029, BT3010, HD2029, HD2091, HD2105, RL4601, RL4604, RL4641, BD3311, AL4810</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Poznámka / kontrola</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>pevné samoobslužné schránky AM či RF (Double, Single, Triple Protection Box Wrap, Alarm Box) s magnetickým zámkem. Dále se jedná o pevné samoobslužné štítky s magnetickým kabelovým zámkem. Určeno k ochraně zboží proti krádeži v obchodech. | štítky AM nebo RF s ocelovým nebo plastovým kabelem, používané především k ochraně lahví, plechovek. Štítky mají standartní pevnost a disponují magnetickým zámkem. Určeno k ochraně zboží proti krádeži v obchodech. | radiofrekvenční nebo akustomagnetické tvrdé etikety s inkoustem uvnitř, sloužící k zabezpečení zboží proti krádeži | standartní tvrdé etikety (štítky) k ochraně textilu, oděvu a příslušenství – frekvenční technologie RF / AM / RF &amp; AM a magnetický zámek. Určeno k ochraně zboží proti krádeži v obchodech.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>AS1029, BT3010, HD2029, HD2091, HD2105, HD2071, BD3311</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n">
-        <v>6627700</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>3972.9</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>4354.087</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>38586.2</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>2,2 %</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="G13" s="5" t="n">
+        <v>128700</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>1104.1</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>1222.571</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>5692.9</v>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Nepodléhá (kap. 85)</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr">
-        <is>
-          <t>CO: pasivní ochranné štítky a etikety EAS (AM 58 kHz, RF 8,2 MHz), fungují jen ve spojení s detekčními branami. Z ČEHO: plastové pouzdro + rezonátor (feritová cívka / magnetostrikční pásek / LC obvod z hliníkové fólie na papíře), ocelový trn/lanko. K ČEMU: ochrana zboží proti krádeži – část poplachového systému. Třída XVI, kap. 85 (pozn. kap. neslučují) → čísl. 8531 (elektrická signalizační zařízení, poplachová zařízení proti vloupání) → 8531 90 části → KN 8531 90 85 ostatní. VPV 1 + 6; u štítků s lankem (CLK872, HDL033, HDL610) podstatný charakter dává štítek (VPV 3b).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ CCT/VPV KN tariff rule (odvozeno)</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>DT052: SUPER COUNTER; DT054: DOME DETACHER; SENSORMATIC SUPER TAG HAND DETACHER WITHOUT LOGO; SUPER DETACHER WITH LANYARD, WITH LID AND KEY; DT4121 MULTI-FUNCTION DETACHER SUPER DETACHER(10000GS)+S3 DETACHER BLACK BLACK; OPTICAL TAG DETACHER-8000GS</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Permanentní magnety z kovu – magnetické odjišťovače (detachery) ochranných štítků</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>DT4010, DT4013, DT4052, DT4086-1, DT4121, DT4096-2</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Ověřit platnost 10místného kódu v TARIC – KN 8531 90 se dále člení (můj původní návrh: 8531 90 85 00). Stop lock HD2071 (HD740) zahrnut pod skupinu HD dle instrukce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>8505 90 29 99</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>měkké akustomagnetické etikety (se semimagnetickým proužkem uvnitř) – s natištěným falešným čárovým kódem, bílé či černé. Jsou určeny k ochraně zboží proti krádeži, často jsou přilepeny na zboží, některé typy jsou vhazovací bez lepidla.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>AL4810</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="H13" s="9" t="n">
-        <v>223</v>
-      </c>
-      <c r="I13" s="10" t="n">
-        <v>89.40000000000001</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>96.914</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>2874</v>
-      </c>
-      <c r="L13" s="8" t="inlineStr">
-        <is>
-          <t>2,2 %</t>
-        </is>
-      </c>
-      <c r="M13" s="8" t="inlineStr">
+      <c r="G14" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>535</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>577.601</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>5500</v>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="N13" s="8" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="O13" s="8" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Nepodléhá (kap. 85)</t>
         </is>
       </c>
-      <c r="P13" s="8" t="inlineStr">
-        <is>
-          <t>CO: odjišťovače (detachery) ochranných štítků – stolní, kopulovitý, ruční. Z ČEHO: silný permanentní magnet (NdFeB, 8000–10000 Gs) v kovovém/plastovém pouzdře. K ČEMU: magnetické uvolnění zámku štítku na pokladně. Třída XVI, kap. 85 → čísl. 8505 (permanentní magnety) → 8505 11 00 z kovu. DT4121 má navíc mechanický S3 odjišťovač – podstatný charakter magnet (VPV 3b). Alternativa: 8531 90 85 (část EAS) – NEJISTÉ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>7326200000</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>⚠️ CCT/VPV KN tariff rule (odvozeno)</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>LD046: LANYARD BLACK CABLE LENGTH 175MM 16MM GROOVED PIN</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>Výrobky z drátu ze železa nebo oceli – ocelová lanka (lanyard) s trnem pro ochranné štítky</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Liší se od mého původního návrhu (8531 90 85 00 – část EAS systému). Ověřit platnost kódu v TARIC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>8534 00 19 00</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>MĚKKÝ PLASTOVÝ ŠTÍTEK RF S POPLACHOVÝM ZABEZPEČENÍM OBSAHUJÍCÍ TIŠTĚNÝ OBVOD, s falešným čárovým kódem, bílá nebo černý</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>RL4601, RL4604, RL4641</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>2339.5</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>2560.356</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>27440</v>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Ne</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Neidentifikováno (ověřit v TARIC)</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Nepodléhá (kap. 85)</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Liší se od mého původního návrhu (8531 90 85 00). Dle instrukce klienta – tištěný obvod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>8505 11 10</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>magnetický oddělovač pro pevný štítek zboží v obchodech</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>DT4010, DT4013, DT4086-1, DT4121, DT4096-2</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>193</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>81.273</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>2574</v>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Ne</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Neidentifikováno (ověřit v TARIC)</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Nepodléhá (kap. 85)</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ Klient uvedl jen 8 míst – doplnit 10místný TARIC kód. Odpovídá mému návrhu (8505 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>8203 20 00 00</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>speciální ruční uvolňovač - kleště- určený k uvolňování pevných štítků AM typu sensormatic (uvolňovač není magnetický)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>DT4052</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>15.641</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Ne</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Neidentifikováno (ověřit v TARIC)</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>Nepodléhá (kap. 82)</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>Ruční kleště, nemagnetický uvolňovač – samostatný kód dle instrukce (můj návrh 8505 11 byl pro tuto položku chybný).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>7312 90 00 00</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>ocelová nebo poplastová lanka sloužící k připojení etikety ke zboží, např. provlečením</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>LD3603</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="G18" s="13" t="n">
         <v>200000</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="H18" s="14" t="n">
         <v>344</v>
       </c>
-      <c r="J14" s="14" t="n">
+      <c r="I18" s="14" t="n">
         <v>376.207</v>
       </c>
-      <c r="K14" s="15" t="n">
+      <c r="J18" s="15" t="n">
         <v>3640</v>
       </c>
-      <c r="L14" s="12" t="inlineStr">
-        <is>
-          <t>1,7 %</t>
-        </is>
-      </c>
-      <c r="M14" s="12" t="inlineStr">
-        <is>
-          <t>ANO – CBAM zboží (7326)</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>Ne pro 7326. Pozor: při zařazení do 7312 AD clo na ocelová lana z CN (60,4 %) – jen průměr &gt; 3 mm.</t>
-        </is>
-      </c>
-      <c r="O14" s="12" t="inlineStr">
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>Ne (7312 není v příloze I CBAM)</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>Ne – AD clo na ocelová lana z ČLR se týká jen 7312 10 (ověřit v TARIC)</t>
+        </is>
+      </c>
+      <c r="M18" s="12" t="inlineStr">
         <is>
           <t>ANO – ocel, kap. 73 → nutná země tavby a odlití + hutní atest</t>
         </is>
       </c>
-      <c r="P14" s="12" t="inlineStr">
-        <is>
-          <t>CO: lanko (lanyard) 175 mm s drážkovaným trnem 16 mm pro připevnění ochranného štítku. Z ČEHO: ocelové lanko s plastovou izolací + ocelový trn. K ČEMU: připevnění štítku k zboží. Samo neobsahuje rezonátor → není částí 8531. Třída XV, kap. 73 → lanko upravené do výrobku s koncovkami → 7326 20 00 výrobky z drátu ze železa/oceli (vyloučení z 7312, VPV 1). Statement dodavatele sám potvrzuje zboží kap. 72/73.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>3926909790</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ CCT/VPV KN tariff rule (odvozeno)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>HD740: STOP LOCK NORMAL LOCK BLACK</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Ostatní výrobky z plastů – plastové zarážky (stop lock) na háčky</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>HD2071</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>Liší se od mého původního návrhu (7326 20 00 00 = CBAM zboží). S kódem klienta 7312 90 CBAM odpadá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>3926 90 97 90 ???</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Instrukce klienta 18.9.2026</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>pojistné kovové víčko (hliník + železo) s aretačním prvkem a kličkou, určené k zakrytí a mechanickému zajištění magnetického uvolňovače pevných bezpečnostních štítků proti krádeži</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>DL4402</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="H15" s="9" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I15" s="10" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>6.441</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>6,5 %</t>
-        </is>
-      </c>
-      <c r="M15" s="8" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>Neidentifikováno (ověřit v TARIC)</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>Nepodléhá (kap. 39)</t>
-        </is>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>CO: „stop lock“ – zarážka na prezentační háček (zabraňuje sejmutí zboží), bez EAS rezonátoru. Z ČEHO: plast + malý kovový magnetický zámek. K ČEMU: mechanická ochrana zboží na háčcích. Podstatný charakter plast (VPV 3b) → třída VII, kap. 39 → 3926 90 97. NEJISTÉ – pokud obsahuje AM/RF prvek, patří do 8531 90 85.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>NEZAŘAZENO</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ nelze zařadit – chybí popis</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>DL4402</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>— (chybí popis zboží)</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>DL4402</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="H16" s="17" t="n">
+      <c r="G19" s="17" t="n">
         <v>60</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="H19" s="18" t="n">
         <v>1.7</v>
       </c>
-      <c r="J16" s="18" t="n">
+      <c r="I19" s="18" t="n">
         <v>2.351</v>
       </c>
-      <c r="K16" s="19" t="n">
+      <c r="J19" s="19" t="n">
         <v>171.6</v>
       </c>
-      <c r="L16" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M16" s="16" t="inlineStr">
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>? (pokud 7616/7326 → ANO)</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="N16" s="16" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="O16" s="16" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="P16" s="16" t="inlineStr">
-        <is>
-          <t>Na faktuře i packing listu je pouze kód „DL4402“ bez popisu (60 ks, 28 g/ks, 2,86 EUR/ks). Nelze odpovědět na CO TO JE / Z ČEHO / K ČEMU → nelze zařadit. Vyžádat popis od dodavatele / klienta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>CELKEM</t>
-        </is>
-      </c>
-      <c r="H17" s="20" t="n">
-        <v>6828983</v>
-      </c>
-      <c r="I17" s="21" t="n">
-        <v>4413.7</v>
-      </c>
-      <c r="J17" s="21" t="n">
-        <v>4836</v>
-      </c>
-      <c r="K17" s="22" t="n">
-        <v>45318.5</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>🟠 ORANŽOVÁ</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>CBAM zboží + melt &amp; pour (ocel) – lanka 7326 20 00</t>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>? (obsahuje železo – pokud kap. 73 → ANO)</t>
+        </is>
+      </c>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ Klient kód sám nepotvrdil („???“). Rozpor: popis uvádí KOVOVÉ víčko (hliník + železo), ale 3926 = výrobky z PLASTŮ. Zařazení vyjasnit (příp. customs.tariff@mauriceward.com).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>🟡 ŽLUTÁ</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Zařazení nejisté – ověřit (případně konzultovat customs.tariff@mauriceward.com)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>🔴 ČERVENÁ</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Položka bez popisu – nelze zařadit (DL4402)</t>
-        </is>
+          <t>CELKEM</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="n">
+        <v>6828983</v>
+      </c>
+      <c r="H20" s="21" t="n">
+        <v>4413.7</v>
+      </c>
+      <c r="I20" s="21" t="n">
+        <v>4836</v>
+      </c>
+      <c r="J20" s="22" t="n">
+        <v>45318.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost</t>
+          <t>🟠 ORANŽOVÁ</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Hmotnost kartonů dle PL + palety (105,50 kg) rozpočítány proporcionálně, faktor 1.022302 → celkem 4 836,00 kg = B/L</t>
+          <t>Ocel kap. 73 – melt &amp; pour (chybí hutní atest) – lanka 7312 90 00 00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HS kódy</t>
+          <t>🟡 ŽLUTÁ</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ŽÁDNÝ HS kód nebyl ve zdrojových dokladech – všechny kódy odvozeny CCT/VPV KN tariff rule. 10místné TARIC přípony ověřit v TARIC při podání JSD.</t>
+          <t>Kód klienta k ověření v TARIC / liší se od mého původního návrhu</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>🔴 ČERVENÁ</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DL4402 – klient kód nepotvrdil (???), rozpor: kovové víčko vs. kód pro plasty</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Hmotnost kartonů dle PL + palety (105,50 kg) rozpočítány proporcionálně, faktor 1.022302 → celkem 4 836,00 kg = B/L</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Popis</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Klient nezaslal český popis – sloupec D = popis z faktury (EN). Sloupec E je pouze návrh k odsouhlasení.</t>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Český popis převzat doslovně z instrukce klienta (sloučeno víc řádků do jednoho).</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1259,7 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -1215,7 +1281,7 @@
       </c>
       <c r="C1" s="23" t="inlineStr">
         <is>
-          <t>Popis (faktura)</t>
+          <t>Popis (faktura EN)</t>
         </is>
       </c>
       <c r="D1" s="23" t="inlineStr">
@@ -1255,842 +1321,842 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>AS1029</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>CLK872: CABLE LOCK-NEW-2A 58KHZ SUPER LOCK BLACK 175MM LENGTH 2 ALARAMS</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="8" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="8" t="n">
         <v>9.404999999999999</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="8" t="n">
         <v>0.86</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="8" t="n">
         <v>172</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>BT3010</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>HDL033-ST: BOTTLE TAG WITH METAL CABLE 160MM 58KHZ SUPER LOCK BLACK 160MM CABLE LENGTH WITH BLACK TUBE, WITH BLACK BALL</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
         <v>2000</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="8" t="n">
         <v>38.4</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="8" t="n">
         <v>40.8</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="8" t="n">
         <v>41.71</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="8" t="n">
         <v>0.1361</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="8" t="n">
         <v>272.2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>DT4010</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>DT052: SUPER COUNTER</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>8505 11 10</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="8" t="n">
         <v>43.2</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="8" t="n">
         <v>44.4</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="8" t="n">
         <v>45.39</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="8" t="n">
         <v>11.8</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="8" t="n">
         <v>1180</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>DT4013</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>DT054: DOME DETACHER</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>8505 11 10</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="8" t="n">
         <v>20.4</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="8" t="n">
         <v>21.468</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="8" t="n">
         <v>14.4</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="8" t="n">
         <v>720</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>DT4052</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>SENSORMATIC SUPER TAG HAND DETACHER WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n">
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>8203 20 00 00</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="8" t="n">
         <v>13.5</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="8" t="n">
         <v>15.3</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="8" t="n">
         <v>15.641</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="8" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>DT4086-1</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>SUPER DETACHER WITH LANYARD, WITH LID AND KEY</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>8505 11 10</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="8" t="n">
         <v>7.4</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="8" t="n">
         <v>8.178000000000001</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="8" t="n">
         <v>15.5</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="8" t="n">
         <v>465</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>DT4121</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>DT4121 MULTI-FUNCTION DETACHER SUPER DETACHER(10000GS)+S3 DETACHER BLACK BLACK</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>8505 11 10</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="8" t="n">
         <v>3.7</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="8" t="n">
         <v>4.3</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="8" t="n">
         <v>4.396</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="8" t="n">
         <v>15.5</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="J8" s="8" t="n">
         <v>155</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>HD2029</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>MINI PENCIL 50*14*20MM NORMAL LOCK 33MM FERRITE 58K GREY</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
         <v>100000</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="8" t="n">
         <v>710</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="8" t="n">
         <v>770</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="8" t="n">
         <v>787.173</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="I9" s="8" t="n">
         <v>0.036</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J9" s="8" t="n">
         <v>3600</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>HD2091</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>HDP674-ST: PICCO 50 8.2MHZ SUPER LOCK WHITE 16MMS</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="8" t="n">
         <v>280</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="8" t="n">
         <v>304</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="H10" s="8" t="n">
         <v>310.78</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I10" s="8" t="n">
         <v>0.0572</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="J10" s="8" t="n">
         <v>1144</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>HD2105</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>HDL610: MICKEY PENCIL-B WITH LANYARD 8.2MHZ SUPER LOCK BLACK CABLE LENGTH 175MM 16MM GROOVED PIN</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n">
         <v>5000</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="H11" s="8" t="n">
         <v>57.249</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="I11" s="8" t="n">
         <v>0.08</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="J11" s="8" t="n">
         <v>400</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>HD2071</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>HD740: STOP LOCK NORMAL LOCK BLACK</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>3926909790</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
         <v>1000</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="F12" s="8" t="n">
         <v>5.7</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="8" t="n">
         <v>6.3</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="H12" s="8" t="n">
         <v>6.441</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="I12" s="8" t="n">
         <v>0.0467</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="J12" s="8" t="n">
         <v>46.7</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>LD3603</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>LD046: LANYARD BLACK CABLE LENGTH 175MM 16MM GROOVED PIN</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>7326200000</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>7312 90 00 00</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n">
         <v>200000</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="8" t="n">
         <v>344</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="8" t="n">
         <v>368</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="8" t="n">
         <v>376.207</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I13" s="8" t="n">
         <v>0.0182</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="J13" s="8" t="n">
         <v>3640</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>RL4601</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 2000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>8534 00 19 00</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
         <v>1000000</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="F14" s="8" t="n">
         <v>460</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="8" t="n">
         <v>490</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="H14" s="8" t="n">
         <v>500.928</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="I14" s="8" t="n">
         <v>0.0048</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="J14" s="8" t="n">
         <v>4800</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>RL4601</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 1000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>8534 00 19 00</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n">
         <v>3000000</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="8" t="n">
         <v>1380</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="8" t="n">
         <v>1470</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="H15" s="8" t="n">
         <v>1502.784</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="I15" s="8" t="n">
         <v>0.0048</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="J15" s="8" t="n">
         <v>14400</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>RL4604</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>PL686: 3*3 ROLL LABEL 8.2MHZ WHITE DEACTIVABLE 1000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>8534 00 19 00</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n">
         <v>1000000</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" s="8" t="n">
         <v>305</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="8" t="n">
         <v>335</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="H16" s="8" t="n">
         <v>342.471</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="I16" s="8" t="n">
         <v>0.0056</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="J16" s="8" t="n">
         <v>5600</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>RL4641</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>ROUND RF LABEL 8.2MHZ WHITE DEACTIVABLE 1000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>8534 00 19 00</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n">
         <v>300000</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" s="8" t="n">
         <v>91.5</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" s="8" t="n">
         <v>100.5</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="H17" s="8" t="n">
         <v>102.741</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="I17" s="8" t="n">
         <v>0.0056</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="J17" s="8" t="n">
         <v>1680</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>RL4601</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 500PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>8534 00 19 00</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n">
         <v>200000</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="F18" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="G18" s="8" t="n">
         <v>109</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="H18" s="8" t="n">
         <v>111.431</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="I18" s="8" t="n">
         <v>0.0048</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="J18" s="8" t="n">
         <v>960</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>BD3311</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>SHELL TAG 58KHZ WHITE SL RED&amp;YELLOW INK(2 RED+1 YELLOW) 16MM SMOOTH PIN</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>8531 90 00 00</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="F19" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" s="8" t="n">
         <v>9.6</v>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="H19" s="8" t="n">
         <v>9.814</v>
       </c>
-      <c r="I19" s="4" t="n">
+      <c r="I19" s="8" t="n">
         <v>0.116</v>
       </c>
-      <c r="J19" s="4" t="n">
+      <c r="J19" s="8" t="n">
         <v>58</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>NEZAŘAZENO</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>3926 90 97 90 ???</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="F20" s="8" t="n">
         <v>1.7</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="8" t="n">
         <v>2.3</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="H20" s="8" t="n">
         <v>2.351</v>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="I20" s="8" t="n">
         <v>2.86</v>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="J20" s="8" t="n">
         <v>171.6</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>AL4810</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>AM LABEL 58KHZ BLACK DEACTIVATABLE</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>8531908500</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>8505 90 29 99</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n">
         <v>1000000</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F21" s="8" t="n">
         <v>535</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="G21" s="8" t="n">
         <v>565</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="H21" s="8" t="n">
         <v>577.601</v>
       </c>
-      <c r="I21" s="4" t="n">
+      <c r="I21" s="8" t="n">
         <v>0.0055</v>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="J21" s="8" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>DT4096-2</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>OPTICAL TAG DETACHER-8000GS</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>8505110000</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n">
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>8505 11 10</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="F22" s="8" t="n">
         <v>1.2</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="G22" s="8" t="n">
         <v>1.8</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="H22" s="8" t="n">
         <v>1.84</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="I22" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="J22" s="8" t="n">
         <v>54</v>
       </c>
     </row>
@@ -2190,159 +2256,159 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>✓ Instrukce klienta s HS kódy a CZ popisy – instrukce_18.9.2026.xlsx (Kateřina Buckingham)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2">
-        <f>== ⚠️ HS KÓDY – CCT/VPV KN tariff rule ===</f>
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <f>== HS KÓDY – dle instrukce klienta ===</f>
         <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Žádná položka neměla HS kód. Všechny kódy odvozeny CCT/VPV KN tariff rule (viz sloupec P v HS Summary):</t>
-        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8531 90 85 00 – EAS štítky a etikety: AS1029, BT3010, HD2029, HD2091, HD2105, BD3311, RL4601, RL4604, RL4641, AL4810</t>
+          <t xml:space="preserve">  8531 90 00 00 – AS1029, BT3010, BD3311, HD2029, HD2091, HD2105, HD2071 (ověřit 10místný kód v TARIC)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8505 11 00 00 – magnetické odjišťovače: DT4010, DT4013, DT4052, DT4086-1, DT4121, DT4096-2  (nejisté – alternativa 8531 90 85)</t>
+          <t xml:space="preserve">  8505 90 29 99 – AL4810</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  7326 20 00 00 – ocelová lanka LD3603  (alternativa 7312 – pozor na AD clo)</t>
+          <t xml:space="preserve">  8534 00 19 00 – RL4601, RL4604, RL4641</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3926 90 97 90 – stop lock HD2071  (nejisté – pokud obsahuje EAS prvek → 8531 90 85)</t>
+          <t xml:space="preserve">  8505 11 10 – DT4010, DT4013, DT4086-1, DT4121, DT4096-2 (⚠️ jen 8 míst – doplnit TARIC)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DL4402 – NEZAŘAZENO, chybí popis → vyžádat od dodavatele</t>
+          <t xml:space="preserve">  8203 20 00 00 – DT4052 (ruční kleště, nemagnetický)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nejisté položky lze konzultovat s customs.tariff@mauriceward.com.</t>
+          <t xml:space="preserve">  7312 90 00 00 – LD3603</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3926 90 97 90 ??? – DL4402 (⚠️ klient nepotvrdil; popis = kovové víčko hliník + železo → kód pro plasty nesedí)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CCT/VPV KN tariff rule již není použit – všechny HS kódy pocházejí z instrukce klienta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
         <f>== POPIS ZBOŽÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Klient nezaslal český popis zboží. V souhrnu použit popis z faktury (EN); navržený CZ popis je pouze návrh.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="2">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Český popis převzat doslovně z instrukce klienta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2">
         <f>== INCOTERM ===</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>CFR Prague (CFR Praha) – na faktuře v poli PAYMENT TERM. Pozn.: CFR je doložka pro námořní dopravu, zde použita pro železnici.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Celní hodnota: cena obsahuje dopravu až do Prahy; náklady na dopravu po vstupu do EU lze odečíst jen pokud jsou doloženy odděleně. Pojištění není uvedeno.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2">
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
         <f>== PREFERENČNÍ PŮVOD / REX ===</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Preferenční věta: NENÍ – v dokladech není žádné prohlášení o preferenčním původu. Čína nemá s EU preferenční dohodu → běžné clo třetí země.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>REX číslo: NENÍ uvedeno na faktuře.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2">
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
         <f>== CBAM ===</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Dotčený HS kód: 7326 20 00 00 (ocelová lanka LD3603) – 344,00 kg NW.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Příjemce V-TOP EUROPE s.r.o. NALEZEN v CBAM_receivers_CZ.xlsx: EORI CZ25795040, Y KÓD = Y137 (do 50 t ročně).</t>
-        </is>
-      </c>
-    </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  povolení (Y128): není; podaná žádost (Y238): není; datum vydání: neuvedeno; ve sloupci H (bez záhlaví) uvedeno: 25MWCCCIM008782.</t>
+          <t>Dle kódů klienta žádná položka není CBAM zboží (7312 90 není v příloze I). Výjimka: DL4402 – pokud by se zařadilo do 7616 (hliník) nebo 7326 (ocel), bylo by CBAM.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>→ Do JSD uvést kód Y137 u HS 7326 20 00 00.</t>
+          <t>Příjemce V-TOP EUROPE s.r.o. je v CBAM_receivers_CZ.xlsx: EORI CZ25795040, Y KÓD = Y137 (do 50 t ročně); povolení ani žádost nejsou; datum vydání neuvedeno; sloupec H: 25MWCCCIM008782.</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2424,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ocelová lanka 7326 20 00 00 (LD3603) – NUTNO doložit zemi tavby a odlití + hutní atest (mill test certificate).</t>
+          <t>Ocelová lanka 7312 90 00 00 (LD3603) – NUTNO doložit zemi tavby a odlití + hutní atest (mill test certificate).</t>
         </is>
       </c>
     </row>
@@ -2372,30 +2438,30 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>DL4402 obsahuje železo – pokud by bylo zařazeno do kap. 73, platí totéž.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Země tavby a odlití ≠ země původu (CN) – evidovat zvlášť.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-    </row>
     <row r="38">
-      <c r="A38" s="2">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2">
         <f>== ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Pro navržené kódy (8531 90 85, 8505 11 00, 7326 20 00, 3926 90 97) nebylo identifikováno antidumpingové clo – ověřit v TARIC.</t>
-        </is>
-      </c>
-    </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pozor: pokud by lanka byla zařazena do 7312 10 (ocelová lana/kabely), platí AD clo na ocelová lana z ČLR (60,4 %) – vztahuje se jen na lana s průřezem &gt; 3 mm.</t>
+          <t>Pro kódy klienta nebylo identifikováno antidumpingové clo – ověřit v TARIC. AD clo na ocelová lana z ČLR se týká 7312 10, ne 7312 90.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V-TOP Europe WPXA26B0912CZ320: classify DL4402 as 7616 99 90 (CBAM)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pg2bih9dX5QihkKn7PSdjY
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
+++ b/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
@@ -41,7 +41,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,18 +131,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -521,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1100,66 +1083,66 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>3926 90 97 90 ???</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>Instrukce klienta 18.9.2026</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>7616 99 90 (TARIC doplnit)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>⚠️ CCT/VPV KN tariff rule – návrh, čeká na potvrzení klienta (klient uvedl 3926 90 97 90 ???)</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>pojistné kovové víčko (hliník + železo) s aretačním prvkem a kličkou, určené k zakrytí a mechanickému zajištění magnetického uvolňovače pevných bezpečnostních štítků proti krádeži</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G19" s="17" t="n">
+      <c r="G19" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="14" t="n">
         <v>1.7</v>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="I19" s="14" t="n">
         <v>2.351</v>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="J19" s="15" t="n">
         <v>171.6</v>
       </c>
-      <c r="K19" s="16" t="inlineStr">
-        <is>
-          <t>? (pokud 7616/7326 → ANO)</t>
-        </is>
-      </c>
-      <c r="L19" s="16" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="M19" s="16" t="inlineStr">
-        <is>
-          <t>? (obsahuje železo – pokud kap. 73 → ANO)</t>
-        </is>
-      </c>
-      <c r="N19" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ Klient kód sám nepotvrdil („???“). Rozpor: popis uvádí KOVOVÉ víčko (hliník + železo), ale 3926 = výrobky z PLASTŮ. Zařazení vyjasnit (příp. customs.tariff@mauriceward.com).</t>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>ANO – CBAM zboží (7616), V-TOP: Y137</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>Neidentifikováno (ověřit v TARIC)</t>
+        </is>
+      </c>
+      <c r="M19" s="12" t="inlineStr">
+        <is>
+          <t>Nepodléhá (hliník). Pokud by převažovalo železo → 7326 90 98 → ANO</t>
+        </is>
+      </c>
+      <c r="N19" s="12" t="inlineStr">
+        <is>
+          <t>Kód klienta 3926 (plasty) nesedí – zboží je kovové. Katalog Ontime: DL4402 = „DETACHER LID“, Ø21×34 mm, T-klička, bez zámku na klíč → ne 8301. Kombinace kovů → převažující kov (pozn. 7 k třídě XV); 28 g/ks odpovídá převážně hliníku → 7616 99 90. Alternativa 7326 90 98, pokud převažuje železo.</t>
         </is>
       </c>
     </row>
@@ -1169,16 +1152,16 @@
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="G20" s="20" t="n">
+      <c r="G20" s="16" t="n">
         <v>6828983</v>
       </c>
-      <c r="H20" s="21" t="n">
+      <c r="H20" s="17" t="n">
         <v>4413.7</v>
       </c>
-      <c r="I20" s="21" t="n">
+      <c r="I20" s="17" t="n">
         <v>4836</v>
       </c>
-      <c r="J20" s="22" t="n">
+      <c r="J20" s="18" t="n">
         <v>45318.5</v>
       </c>
     </row>
@@ -1190,7 +1173,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ocel kap. 73 – melt &amp; pour (chybí hutní atest) – lanka 7312 90 00 00</t>
+          <t>LD3603: ocel kap. 73 – melt &amp; pour (chybí hutní atest). DL4402: CBAM zboží (7616) – kód navržen, čeká na potvrzení klienta</t>
         </is>
       </c>
     </row>
@@ -1209,34 +1192,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>🔴 ČERVENÁ</t>
+          <t>Hrubá hmotnost</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DL4402 – klient kód nepotvrdil (???), rozpor: kovové víčko vs. kód pro plasty</t>
+          <t>Hmotnost kartonů dle PL + palety (105,50 kg) rozpočítány proporcionálně, faktor 1.022302 → celkem 4 836,00 kg = B/L</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost</t>
+          <t>Popis</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
-        <is>
-          <t>Hmotnost kartonů dle PL + palety (105,50 kg) rozpočítány proporcionálně, faktor 1.022302 → celkem 4 836,00 kg = B/L</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Popis</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
         <is>
           <t>Český popis převzat doslovně z instrukce klienta (sloučeno víc řádků do jednoho).</t>
         </is>
@@ -1269,52 +1240,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Odesílatel</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Ontime kód</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="19" t="inlineStr">
         <is>
           <t>Popis (faktura EN)</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D1" s="19" t="inlineStr">
         <is>
           <t>HS kód (TARIC)</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="19" t="inlineStr">
         <is>
           <t>Množství (ks)</t>
         </is>
       </c>
-      <c r="F1" s="23" t="inlineStr">
+      <c r="F1" s="19" t="inlineStr">
         <is>
           <t>Čistá hm. (kg)</t>
         </is>
       </c>
-      <c r="G1" s="23" t="inlineStr">
+      <c r="G1" s="19" t="inlineStr">
         <is>
           <t>Hrubá hm. kartony (kg)</t>
         </is>
       </c>
-      <c r="H1" s="23" t="inlineStr">
+      <c r="H1" s="19" t="inlineStr">
         <is>
           <t>Hrubá hm. vč. palet (kg)</t>
         </is>
       </c>
-      <c r="I1" s="23" t="inlineStr">
+      <c r="I1" s="19" t="inlineStr">
         <is>
           <t>Cena/ks EUR</t>
         </is>
       </c>
-      <c r="J1" s="23" t="inlineStr">
+      <c r="J1" s="19" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
@@ -2058,7 +2029,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>3926 90 97 90 ???</t>
+          <t>7616 99 90 (TARIC doplnit)</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
@@ -2215,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -2316,173 +2287,180 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3926 90 97 90 ??? – DL4402 (⚠️ klient nepotvrdil; popis = kovové víčko hliník + železo → kód pro plasty nesedí)</t>
+          <t xml:space="preserve">  ⚠️ 7616 99 90 – DL4402 – zařazeno CCT/VPV KN tariff rule (klient uvedl 3926 90 97 90 ???, což nesedí – kovové víčko hliník + železo). Čeká na potvrzení Kateřiny.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CCT/VPV KN tariff rule již není použit – všechny HS kódy pocházejí z instrukce klienta.</t>
+          <t xml:space="preserve">     Katalog Ontime: DL4402 = DETACHER LID, Ø21×34 mm, T-klička, bez klíče (ne 8301). Převažující kov dle hmotnosti (28 g/ks) = hliník → 7616 99 90; alternativa 7326 90 98.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ostatní HS kódy pocházejí z instrukce klienta.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
         <f>== POPIS ZBOŽÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Český popis převzat doslovně z instrukce klienta.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
         <f>== INCOTERM ===</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>CFR Prague (CFR Praha) – na faktuře v poli PAYMENT TERM. Pozn.: CFR je doložka pro námořní dopravu, zde použita pro železnici.</t>
-        </is>
-      </c>
-    </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>CFR Prague (CFR Praha) – na faktuře v poli PAYMENT TERM. Pozn.: CFR je doložka pro námořní dopravu, zde použita pro železnici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Celní hodnota: cena obsahuje dopravu až do Prahy; náklady na dopravu po vstupu do EU lze odečíst jen pokud jsou doloženy odděleně. Pojištění není uvedeno.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="2">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2">
         <f>== PREFERENČNÍ PŮVOD / REX ===</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Preferenční věta: NENÍ – v dokladech není žádné prohlášení o preferenčním původu. Čína nemá s EU preferenční dohodu → běžné clo třetí země.</t>
-        </is>
-      </c>
-    </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Preferenční věta: NENÍ – v dokladech není žádné prohlášení o preferenčním původu. Čína nemá s EU preferenční dohodu → běžné clo třetí země.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>REX číslo: NENÍ uvedeno na faktuře.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="2">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2">
         <f>== CBAM ===</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Dle kódů klienta žádná položka není CBAM zboží (7312 90 není v příloze I). Výjimka: DL4402 – pokud by se zařadilo do 7616 (hliník) nebo 7326 (ocel), bylo by CBAM.</t>
-        </is>
-      </c>
-    </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>CBAM zboží: DL4402 – 7616 99 90 (hliník), 60 ks, 1,70 kg NW → do JSD uvést Y137. Ostatní kódy klienta nejsou CBAM (7312 90 není v příloze I).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Příjemce V-TOP EUROPE s.r.o. je v CBAM_receivers_CZ.xlsx: EORI CZ25795040, Y KÓD = Y137 (do 50 t ročně); povolení ani žádost nejsou; datum vydání neuvedeno; sloupec H: 25MWCCCIM008782.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="A33" s="2">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2">
         <f>== MELT AND POUR (země tavby a odlití) ===</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Ocelová lanka 7312 90 00 00 (LD3603) – NUTNO doložit zemi tavby a odlití + hutní atest (mill test certificate).</t>
-        </is>
-      </c>
-    </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>V dokladech CHYBÍ – statement dodavatele řeší jen ruský původ (sankce), zemi tavby a odlití neuvádí. → Vyžádat hutní atest před proclením.</t>
+          <t>Ocelová lanka 7312 90 00 00 (LD3603) – NUTNO doložit zemi tavby a odlití + hutní atest (mill test certificate).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL4402 obsahuje železo – pokud by bylo zařazeno do kap. 73, platí totéž.</t>
+          <t>V dokladech CHYBÍ – statement dodavatele řeší jen ruský původ (sankce), zemi tavby a odlití neuvádí. → Vyžádat hutní atest před proclením.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>DL4402 zařazeno jako hliník (7616) – melt &amp; pour se netýká. Pokud by bylo nakonec 7326 (ocel), platí totéž co u lanek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Země tavby a odlití ≠ země původu (CN) – evidovat zvlášť.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" s="2">
+      <c r="A39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2">
         <f>== ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Pro kódy klienta nebylo identifikováno antidumpingové clo – ověřit v TARIC. AD clo na ocelová lana z ČLR se týká 7312 10, ne 7312 90.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-    </row>
     <row r="42">
-      <c r="A42" s="2">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2">
         <f>== HMOTNOSTI ===</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Čistá hmotnost celkem: 4 413,70 kg (PL). Hrubá hmotnost celkem: 4 836,00 kg (PL + B/L) = kartony 4 730,50 kg + 7 palet 105,50 kg.</t>
-        </is>
-      </c>
-    </row>
     <row r="44">
       <c r="A44" t="inlineStr">
+        <is>
+          <t>Čistá hmotnost celkem: 4 413,70 kg (PL). Hrubá hmotnost celkem: 4 836,00 kg (PL + B/L) = kartony 4 730,50 kg + 7 palet 105,50 kg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Hrubá hmotnost na HS kód: kartony dle PL + palety rozpočítány proporcionálně.</t>
         </is>

</xml_diff>

<commit_message>
V-TOP Europe WPXA26B0912CZ320: drop 7326 alternative for DL4402, separate row colours
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pg2bih9dX5QihkKn7PSdjY
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
+++ b/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
@@ -1078,71 +1078,71 @@
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>Liší se od mého původního návrhu (7326 20 00 00 = CBAM zboží). S kódem klienta 7312 90 CBAM odpadá.</t>
+          <t>Dle instrukce klienta. 7312 90 není CBAM zboží.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>7616 99 90 (TARIC doplnit)</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>⚠️ CCT/VPV KN tariff rule – návrh, čeká na potvrzení klienta (klient uvedl 3926 90 97 90 ???)</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>pojistné kovové víčko (hliník + železo) s aretačním prvkem a kličkou, určené k zakrytí a mechanickému zajištění magnetického uvolňovače pevných bezpečnostních štítků proti krádeži</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="G19" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="H19" s="14" t="n">
+      <c r="H19" s="6" t="n">
         <v>1.7</v>
       </c>
-      <c r="I19" s="14" t="n">
+      <c r="I19" s="6" t="n">
         <v>2.351</v>
       </c>
-      <c r="J19" s="15" t="n">
+      <c r="J19" s="7" t="n">
         <v>171.6</v>
       </c>
-      <c r="K19" s="12" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>ANO – CBAM zboží (7616), V-TOP: Y137</t>
         </is>
       </c>
-      <c r="L19" s="12" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="M19" s="12" t="inlineStr">
-        <is>
-          <t>Nepodléhá (hliník). Pokud by převažovalo železo → 7326 90 98 → ANO</t>
-        </is>
-      </c>
-      <c r="N19" s="12" t="inlineStr">
-        <is>
-          <t>Kód klienta 3926 (plasty) nesedí – zboží je kovové. Katalog Ontime: DL4402 = „DETACHER LID“, Ø21×34 mm, T-klička, bez zámku na klíč → ne 8301. Kombinace kovů → převažující kov (pozn. 7 k třídě XV); 28 g/ks odpovídá převážně hliníku → 7616 99 90. Alternativa 7326 90 98, pokud převažuje železo.</t>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Nepodléhá (hliník, kap. 76)</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Kód klienta 3926 (plasty) nesedí – zboží je kovové. Katalog Ontime: DL4402 = „DETACHER LID“, Ø21×34 mm, T-klička, bez zámku na klíč → ne 8301. Kombinace kovů → převažující kov (pozn. 7 k třídě XV); 28 g/ks odpovídá převážně hliníku → 7616 99 90.</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>LD3603: ocel kap. 73 – melt &amp; pour (chybí hutní atest). DL4402: CBAM zboží (7616) – kód navržen, čeká na potvrzení klienta</t>
+          <t>LD3603 (lanka) – ocel kap. 73 – melt &amp; pour (chybí hutní atest)</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kód klienta k ověření v TARIC / liší se od mého původního návrhu</t>
+          <t>Kód k ověření v TARIC / liší se od mého původního návrhu. DL4402 (víčko) – kód 7616 99 90 navržen, čeká na potvrzení klienta; CBAM zboží</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Katalog Ontime: DL4402 = DETACHER LID, Ø21×34 mm, T-klička, bez klíče (ne 8301). Převažující kov dle hmotnosti (28 g/ks) = hliník → 7616 99 90; alternativa 7326 90 98.</t>
+          <t xml:space="preserve">     Katalog Ontime: DL4402 = DETACHER LID, Ø21×34 mm, T-klička, bez klíče (ne 8301). Převažující kov dle hmotnosti (28 g/ks) = hliník → 7616 99 90.</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DL4402 zařazeno jako hliník (7616) – melt &amp; pour se netýká. Pokud by bylo nakonec 7326 (ocel), platí totéž co u lanek.</t>
+          <t>DL4402 zařazeno jako hliník (7616) – melt &amp; pour se netýká.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V-TOP Europe WPXA26B0912CZ320: 8531 90 00 00 confirmed, flag 8505 11 10 vs 11 90
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pg2bih9dX5QihkKn7PSdjY
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
+++ b/output/HS_Code_Summary_V_TOP_Europe_WPXA26B0912CZ320.xlsx
@@ -97,6 +97,18 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -107,18 +119,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -758,261 +758,261 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>Ověřit platnost 10místného kódu v TARIC – KN 8531 90 se dále člení (můj původní návrh: 8531 90 85 00). Stop lock HD2071 (HD740) zahrnut pod skupinu HD dle instrukce.</t>
+          <t>Kód platný – ověřeno v celním systému (8531 90 00, DK 00). Stop lock HD2071 (HD740) zahrnut pod skupinu HD dle instrukce.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>8505 90 29 99</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Instrukce klienta 18.9.2026</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>měkké akustomagnetické etikety (se semimagnetickým proužkem uvnitř) – s natištěným falešným čárovým kódem, bílé či černé. Jsou určeny k ochraně zboží proti krádeži, často jsou přilepeny na zboží, některé typy jsou vhazovací bez lepidla.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>AL4810</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="10" t="n">
         <v>535</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="10" t="n">
         <v>577.601</v>
       </c>
-      <c r="J14" s="7" t="n">
+      <c r="J14" s="11" t="n">
         <v>5500</v>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>Nepodléhá (kap. 85)</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>Liší se od mého původního návrhu (8531 90 85 00 – část EAS systému). Ověřit platnost kódu v TARIC.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>8534 00 19 00</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Instrukce klienta 18.9.2026</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>MĚKKÝ PLASTOVÝ ŠTÍTEK RF S POPLACHOVÝM ZABEZPEČENÍM OBSAHUJÍCÍ TIŠTĚNÝ OBVOD, s falešným čárovým kódem, bílá nebo černý</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>RL4601, RL4604, RL4641</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="9" t="n">
         <v>5500000</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="10" t="n">
         <v>2339.5</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="10" t="n">
         <v>2560.356</v>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="J15" s="11" t="n">
         <v>27440</v>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L15" s="8" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>Nepodléhá (kap. 85)</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>Liší se od mého původního návrhu (8531 90 85 00). Dle instrukce klienta – tištěný obvod.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>8505 11 10</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Instrukce klienta 18.9.2026</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>magnetický oddělovač pro pevný štítek zboží v obchodech</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>DT4010, DT4013, DT4086-1, DT4121, DT4096-2</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="G16" s="9" t="n">
         <v>193</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="10" t="n">
         <v>75.90000000000001</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="10" t="n">
         <v>81.273</v>
       </c>
-      <c r="J16" s="7" t="n">
+      <c r="J16" s="11" t="n">
         <v>2574</v>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>Nepodléhá (kap. 85)</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ Klient uvedl jen 8 míst – doplnit 10místný TARIC kód. Odpovídá mému návrhu (8505 11).</t>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>⚠️ ROZPOR: Kateřina uvedla 8505 11 10, v celním systému bylo zadáno 8505 11 90 (DK 99). Ověřit správnou podpoložku 8505 11 xx a doplnit DK.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>8203 20 00 00</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Instrukce klienta 18.9.2026</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>speciální ruční uvolňovač - kleště- určený k uvolňování pevných štítků AM typu sensormatic (uvolňovač není magnetický)</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>DT4052</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="H17" s="10" t="n">
+      <c r="H17" s="6" t="n">
         <v>13.5</v>
       </c>
-      <c r="I17" s="10" t="n">
+      <c r="I17" s="6" t="n">
         <v>15.641</v>
       </c>
-      <c r="J17" s="11" t="n">
+      <c r="J17" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="M17" s="8" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Nepodléhá (kap. 82)</t>
         </is>
       </c>
-      <c r="N17" s="8" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Ruční kleště, nemagnetický uvolňovač – samostatný kód dle instrukce (můj návrh 8505 11 byl pro tuto položku chybný).</t>
         </is>
@@ -1083,64 +1083,64 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>7616 99 90 (TARIC doplnit)</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>⚠️ CCT/VPV KN tariff rule – návrh, čeká na potvrzení klienta (klient uvedl 3926 90 97 90 ???)</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>pojistné kovové víčko (hliník + železo) s aretačním prvkem a kličkou, určené k zakrytí a mechanickému zajištění magnetického uvolňovače pevných bezpečnostních štítků proti krádeži</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="G19" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H19" s="10" t="n">
         <v>1.7</v>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I19" s="10" t="n">
         <v>2.351</v>
       </c>
-      <c r="J19" s="7" t="n">
+      <c r="J19" s="11" t="n">
         <v>171.6</v>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>ANO – CBAM zboží (7616), V-TOP: Y137</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L19" s="8" t="inlineStr">
         <is>
           <t>Neidentifikováno (ověřit v TARIC)</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t>Nepodléhá (hliník, kap. 76)</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="N19" s="8" t="inlineStr">
         <is>
           <t>Kód klienta 3926 (plasty) nesedí – zboží je kovové. Katalog Ontime: DL4402 = „DETACHER LID“, Ø21×34 mm, T-klička, bez zámku na klíč → ne 8301. Kombinace kovů → převažující kov (pozn. 7 k třídě XV); 28 g/ks odpovídá převážně hliníku → 7616 99 90.</t>
         </is>
@@ -1292,842 +1292,842 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>AS1029</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>CLK872: CABLE LOCK-NEW-2A 58KHZ SUPER LOCK BLACK 175MM LENGTH 2 ALARAMS</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="4" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="4" t="n">
         <v>9.404999999999999</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="4" t="n">
         <v>0.86</v>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="J2" s="4" t="n">
         <v>172</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>BT3010</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>HDL033-ST: BOTTLE TAG WITH METAL CABLE 160MM 58KHZ SUPER LOCK BLACK 160MM CABLE LENGTH WITH BLACK TUBE, WITH BLACK BALL</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="4" t="n">
         <v>2000</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="4" t="n">
         <v>38.4</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="4" t="n">
         <v>40.8</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="4" t="n">
         <v>41.71</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="4" t="n">
         <v>0.1361</v>
       </c>
-      <c r="J3" s="8" t="n">
+      <c r="J3" s="4" t="n">
         <v>272.2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>DT4010</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>DT052: SUPER COUNTER</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>8505 11 10</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="4" t="n">
         <v>43.2</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="4" t="n">
         <v>44.4</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="4" t="n">
         <v>45.39</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="4" t="n">
         <v>11.8</v>
       </c>
-      <c r="J4" s="8" t="n">
+      <c r="J4" s="4" t="n">
         <v>1180</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>DT4013</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>DT054: DOME DETACHER</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>8505 11 10</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="4" t="n">
         <v>20.4</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="4" t="n">
         <v>21.468</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="4" t="n">
         <v>14.4</v>
       </c>
-      <c r="J5" s="8" t="n">
+      <c r="J5" s="4" t="n">
         <v>720</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>DT4052</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>SENSORMATIC SUPER TAG HAND DETACHER WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>8203 20 00 00</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="4" t="n">
         <v>13.5</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="4" t="n">
         <v>15.3</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="4" t="n">
         <v>15.641</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="4" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>DT4086-1</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>SUPER DETACHER WITH LANYARD, WITH LID AND KEY</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>8505 11 10</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="4" t="n">
         <v>7.4</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="4" t="n">
         <v>8.178000000000001</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="4" t="n">
         <v>15.5</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="4" t="n">
         <v>465</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>DT4121</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>DT4121 MULTI-FUNCTION DETACHER SUPER DETACHER(10000GS)+S3 DETACHER BLACK BLACK</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>8505 11 10</t>
         </is>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="4" t="n">
         <v>3.7</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="4" t="n">
         <v>4.3</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="4" t="n">
         <v>4.396</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="4" t="n">
         <v>15.5</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="4" t="n">
         <v>155</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>HD2029</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>MINI PENCIL 50*14*20MM NORMAL LOCK 33MM FERRITE 58K GREY</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="4" t="n">
         <v>100000</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="4" t="n">
         <v>710</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="4" t="n">
         <v>770</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="4" t="n">
         <v>787.173</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="4" t="n">
         <v>0.036</v>
       </c>
-      <c r="J9" s="8" t="n">
+      <c r="J9" s="4" t="n">
         <v>3600</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>HD2091</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>HDP674-ST: PICCO 50 8.2MHZ SUPER LOCK WHITE 16MMS</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="4" t="n">
         <v>20000</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="4" t="n">
         <v>304</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="4" t="n">
         <v>310.78</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="4" t="n">
         <v>0.0572</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="4" t="n">
         <v>1144</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>HD2105</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>HDL610: MICKEY PENCIL-B WITH LANYARD 8.2MHZ SUPER LOCK BLACK CABLE LENGTH 175MM 16MM GROOVED PIN</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="4" t="n">
         <v>5000</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="4" t="n">
         <v>57.249</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="4" t="n">
         <v>0.08</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J11" s="4" t="n">
         <v>400</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>HD2071</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>HD740: STOP LOCK NORMAL LOCK BLACK</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="4" t="n">
         <v>5.7</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="4" t="n">
         <v>6.441</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="4" t="n">
         <v>0.0467</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="J12" s="4" t="n">
         <v>46.7</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>LD3603</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>LD046: LANYARD BLACK CABLE LENGTH 175MM 16MM GROOVED PIN</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>7312 90 00 00</t>
         </is>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="4" t="n">
         <v>200000</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="4" t="n">
         <v>344</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="4" t="n">
         <v>368</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="4" t="n">
         <v>376.207</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="4" t="n">
         <v>0.0182</v>
       </c>
-      <c r="J13" s="8" t="n">
+      <c r="J13" s="4" t="n">
         <v>3640</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>RL4601</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 2000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>8534 00 19 00</t>
         </is>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="4" t="n">
         <v>1000000</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="4" t="n">
         <v>460</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="4" t="n">
         <v>490</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="4" t="n">
         <v>500.928</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="4" t="n">
         <v>0.0048</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="4" t="n">
         <v>4800</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>RL4601</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 1000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>8534 00 19 00</t>
         </is>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="4" t="n">
         <v>3000000</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="4" t="n">
         <v>1380</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="4" t="n">
         <v>1470</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="4" t="n">
         <v>1502.784</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="4" t="n">
         <v>0.0048</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="4" t="n">
         <v>14400</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>RL4604</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>PL686: 3*3 ROLL LABEL 8.2MHZ WHITE DEACTIVABLE 1000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>8534 00 19 00</t>
         </is>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="4" t="n">
         <v>1000000</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="4" t="n">
         <v>305</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="4" t="n">
         <v>335</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="4" t="n">
         <v>342.471</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="4" t="n">
         <v>0.0056</v>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J16" s="4" t="n">
         <v>5600</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>RL4641</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>ROUND RF LABEL 8.2MHZ WHITE DEACTIVABLE 1000PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>8534 00 19 00</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="4" t="n">
         <v>300000</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="4" t="n">
         <v>91.5</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="4" t="n">
         <v>100.5</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="4" t="n">
         <v>102.741</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="4" t="n">
         <v>0.0056</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="J17" s="4" t="n">
         <v>1680</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>RL4601</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>PL519: ROLL LABELS 8.2MHZ BARCODE DEACTIVABLE 40*40MM 500PCS PER ROLL WITHOUT LOGO</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>8534 00 19 00</t>
         </is>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="4" t="n">
         <v>200000</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="4" t="n">
         <v>103</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="4" t="n">
         <v>111.431</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="4" t="n">
         <v>0.0048</v>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="J18" s="4" t="n">
         <v>960</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>BD3311</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>SHELL TAG 58KHZ WHITE SL RED&amp;YELLOW INK(2 RED+1 YELLOW) 16MM SMOOTH PIN</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>8531 90 00 00</t>
         </is>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="4" t="n">
         <v>500</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="4" t="n">
         <v>9.6</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="4" t="n">
         <v>9.814</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="4" t="n">
         <v>0.116</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="4" t="n">
         <v>58</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>DL4402</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>7616 99 90 (TARIC doplnit)</t>
         </is>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="4" t="n">
         <v>2.3</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="4" t="n">
         <v>2.351</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="4" t="n">
         <v>2.86</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="4" t="n">
         <v>171.6</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>AL4810</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>AM LABEL 58KHZ BLACK DEACTIVATABLE</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>8505 90 29 99</t>
         </is>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="4" t="n">
         <v>1000000</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="4" t="n">
         <v>535</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="4" t="n">
         <v>565</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="4" t="n">
         <v>577.601</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="4" t="n">
         <v>0.0055</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>HANGZHOU ONTIME I.T. CO., LTD. (CN)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>DT4096-2</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>OPTICAL TAG DETACHER-8000GS</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>8505 11 10</t>
         </is>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="4" t="n">
         <v>1.2</v>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="4" t="n">
         <v>1.8</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="4" t="n">
         <v>1.84</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J22" s="4" t="n">
         <v>54</v>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8531 90 00 00 – AS1029, BT3010, BD3311, HD2029, HD2091, HD2105, HD2071 (ověřit 10místný kód v TARIC)</t>
+          <t xml:space="preserve">  8531 90 00 00 – AS1029, BT3010, BD3311, HD2029, HD2091, HD2105, HD2071 (kód ověřen v celním systému, DK 00)</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8505 11 10 – DT4010, DT4013, DT4086-1, DT4121, DT4096-2 (⚠️ jen 8 míst – doplnit TARIC)</t>
+          <t xml:space="preserve">  8505 11 10 – DT4010, DT4013, DT4086-1, DT4121, DT4096-2 (⚠️ rozpor: v celním systému zadáno 8505 11 90 / DK 99 – ověřit, která podpoložka platí)</t>
         </is>
       </c>
     </row>

</xml_diff>